<commit_message>
images adding from admin to our products page
</commit_message>
<xml_diff>
--- a/suvai-organics/suvai-organics/data/products.xlsx
+++ b/suvai-organics/suvai-organics/data/products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,6 +490,86 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>2025-08-09T22:20:17.899027</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>678669</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>yeshwanth</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>tharkuri</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Seasonal Produce</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>100000000000000</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>a1ee3180ea324906b9105d53fc6c97d2_WIN_20250816_19_03_12_Pro.jpg</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2025-08-16T19:04:30.049811</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sector 41</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COCONUT OIL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Coconut oil is a popular edible oil from the coconut palm, solid below 77°F (25°C) and clear liquid above, known for its distinct coconut scent (unrefined) and high content of medium-chain fatty acids (MCTs), especially lauric acid, making it a skincare moisturizer, cooking fat, and ingredient in cosmetics/soaps, valued for its nourishing properties but often debated regarding health benefits, with virgin oil being unrefined for maximum nutrients.</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cold-pressed Oils</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>516a5be241354489979ea9d4fc5e0be5_COCONUT.jpg</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2025-12-28T20:55:41.455295</t>
         </is>
       </c>
     </row>

</xml_diff>